<commit_message>
Fix GitHub Actions workflows
</commit_message>
<xml_diff>
--- a/test_report.xlsx
+++ b/test_report.xlsx
@@ -538,7 +538,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -904,7 +904,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I401"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>

</xml_diff>